<commit_message>
Upload file on 2-09-2026
</commit_message>
<xml_diff>
--- a/12602441.xlsx
+++ b/12602441.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/565755648f0a3f81/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="8_{F92E2664-E68F-4788-901C-B0B3E7C55010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4211C083-36D5-4EF3-9AD8-64781759248A}"/>
+  <xr:revisionPtr revIDLastSave="179" documentId="8_{F92E2664-E68F-4788-901C-B0B3E7C55010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD9633C5-BBAE-4FD2-9DE1-6F81347C3148}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1629,26 +1629,50 @@
       </c>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B19" s="14">
+        <v>360</v>
+      </c>
+      <c r="C19" s="14">
+        <v>20</v>
+      </c>
+      <c r="D19" s="14">
+        <v>120</v>
+      </c>
+      <c r="E19" s="14">
+        <v>120</v>
+      </c>
+      <c r="F19" s="14">
+        <v>300</v>
+      </c>
+      <c r="G19" s="14">
+        <v>6</v>
+      </c>
+      <c r="H19" s="14">
+        <v>140</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>1060</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
+        <v>380</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="13"/>

</xml_diff>